<commit_message>
planes de clase actualizados al 15 de febrero
</commit_message>
<xml_diff>
--- a/distribucionClases2026_2.xlsx
+++ b/distribucionClases2026_2.xlsx
@@ -43,19 +43,19 @@
     <t xml:space="preserve">Lektion 5</t>
   </si>
   <si>
+    <t xml:space="preserve">Lektion 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23-27 Feb</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lektion 6</t>
   </si>
   <si>
-    <t xml:space="preserve">23-27 Feb</t>
-  </si>
-  <si>
     <t xml:space="preserve">2-5 mar</t>
   </si>
   <si>
     <t xml:space="preserve">Lektion 11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lektion 7</t>
   </si>
   <si>
     <t xml:space="preserve">9-13 mar</t>
@@ -124,6 +124,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -183,8 +184,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -315,220 +320,220 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="0" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="0" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="0" t="s">
+      <c r="D13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="0" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="B7" s="0" t="s">
+      <c r="D14" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C8" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D11" s="0" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>22</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="D12" s="0" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="0" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="B15" s="0" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D15" s="0" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>28</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="1" t="s">
         <v>14</v>
       </c>
     </row>
@@ -537,8 +542,8 @@
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12Página &amp;P</oddFooter>
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Página &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
planes de clase para el viernes 6 de marzo
</commit_message>
<xml_diff>
--- a/distribucionClases2026_2.xlsx
+++ b/distribucionClases2026_2.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="32">
   <si>
     <t xml:space="preserve">Segundo</t>
   </si>
@@ -58,28 +58,34 @@
     <t xml:space="preserve">Lektion 11</t>
   </si>
   <si>
+    <t xml:space="preserve">Lektion 8</t>
+  </si>
+  <si>
     <t xml:space="preserve">9-13 mar</t>
   </si>
   <si>
+    <t xml:space="preserve">Lektion 8/9</t>
+  </si>
+  <si>
     <t xml:space="preserve">16-20 mar</t>
   </si>
   <si>
     <t xml:space="preserve">Lektion 12</t>
   </si>
   <si>
-    <t xml:space="preserve">Lektion 8</t>
+    <t xml:space="preserve">Lektion 9</t>
   </si>
   <si>
     <t xml:space="preserve">23-27 mar</t>
   </si>
   <si>
+    <t xml:space="preserve">Lektion 9/10</t>
+  </si>
+  <si>
     <t xml:space="preserve">6-10 abr</t>
   </si>
   <si>
     <t xml:space="preserve">Lektion 13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lektion 9</t>
   </si>
   <si>
     <t xml:space="preserve">13-17 abr</t>
@@ -380,12 +386,12 @@
         <v>7</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>11</v>
@@ -394,99 +400,99 @@
         <v>7</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="D9" s="1" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>11</v>
@@ -497,44 +503,44 @@
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>